<commit_message>
update to Manu file
</commit_message>
<xml_diff>
--- a/results/02-2025/beta/contributions-02-2025.xlsx
+++ b/results/02-2025/beta/contributions-02-2025.xlsx
@@ -65,7 +65,7 @@
     <t xml:space="preserve">federal_subsidies_contribution</t>
   </si>
   <si>
-    <t xml:space="preserve">federal_aid_to_small_businesses_arp</t>
+    <t xml:space="preserve">federal_aid_to_small_businesses_arp_contribution</t>
   </si>
   <si>
     <t xml:space="preserve">federal_other_direct_aid_arp_contribution</t>
@@ -1335,9 +1335,7 @@
       <c r="O2"/>
       <c r="P2"/>
       <c r="Q2"/>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
+      <c r="R2"/>
       <c r="S2"/>
       <c r="T2"/>
       <c r="U2"/>
@@ -20783,7 +20781,7 @@
         <v>0.482083210091057</v>
       </c>
       <c r="R207" t="n">
-        <v>58.78296</v>
+        <v>0.0479900759427587</v>
       </c>
       <c r="S207" t="n">
         <v>-0.0475990783100114</v>
@@ -20878,7 +20876,7 @@
         <v>0.26753291628999</v>
       </c>
       <c r="R208" t="n">
-        <v>267.78904</v>
+        <v>0.194542041773206</v>
       </c>
       <c r="S208" t="n">
         <v>0.00815216541343598</v>
@@ -20973,7 +20971,7 @@
         <v>0.068285943745188</v>
       </c>
       <c r="R209" t="n">
-        <v>110.248</v>
+        <v>0.0503170157550065</v>
       </c>
       <c r="S209" t="n">
         <v>0.0890272541814862</v>
@@ -21068,7 +21066,7 @@
         <v>-0.142995617838387</v>
       </c>
       <c r="R210" t="n">
-        <v>110.248</v>
+        <v>-0.0367891456962245</v>
       </c>
       <c r="S210" t="n">
         <v>0.0548942288001818</v>
@@ -21163,7 +21161,7 @@
         <v>-0.241839656558443</v>
       </c>
       <c r="R211" t="n">
-        <v>110.248</v>
+        <v>0.0261593640052049</v>
       </c>
       <c r="S211" t="n">
         <v>0.0329717470857747</v>
@@ -21258,7 +21256,7 @@
         <v>-0.202382302123556</v>
       </c>
       <c r="R212" t="n">
-        <v>110.248</v>
+        <v>0.0258982918675242</v>
       </c>
       <c r="S212" t="n">
         <v>-0.0655652053829996</v>
@@ -21353,7 +21351,7 @@
         <v>-0.10036732151305</v>
       </c>
       <c r="R213" t="n">
-        <v>12.726</v>
+        <v>-0.0365304709791591</v>
       </c>
       <c r="S213" t="n">
         <v>-0.0657472149902382</v>
@@ -21448,7 +21446,7 @@
         <v>-0.0826792024111309</v>
       </c>
       <c r="R214" t="n">
-        <v>12.726</v>
+        <v>-0.036304584635801</v>
       </c>
       <c r="S214" t="n">
         <v>-0.0494052000034905</v>
@@ -21543,7 +21541,7 @@
         <v>-0.360000097756315</v>
       </c>
       <c r="R215" t="n">
-        <v>12.726</v>
+        <v>0.000539751927453967</v>
       </c>
       <c r="S215" t="n">
         <v>-0.0417113484797409</v>
@@ -21638,7 +21636,7 @@
         <v>-0.374991548534942</v>
       </c>
       <c r="R216" t="n">
-        <v>12.726</v>
+        <v>0.000608599167464871</v>
       </c>
       <c r="S216" t="n">
         <v>-0.0267320020971429</v>
@@ -21733,7 +21731,7 @@
         <v>-0.162333472688065</v>
       </c>
       <c r="R217" t="n">
-        <v>1.365</v>
+        <v>-0.00565460017451395</v>
       </c>
       <c r="S217" t="n">
         <v>-0.0266258923286068</v>
@@ -21828,7 +21826,7 @@
         <v>-0.142523794737716</v>
       </c>
       <c r="R218" t="n">
-        <v>1.365</v>
+        <v>-0.00648103795740414</v>
       </c>
       <c r="S218" t="n">
         <v>-0.0375809815098436</v>
@@ -21923,7 +21921,7 @@
         <v>-0.339297316804842</v>
       </c>
       <c r="R219" t="n">
-        <v>1.365</v>
+        <v>-0.0166531841273023</v>
       </c>
       <c r="S219" t="n">
         <v>-0.0356906395802881</v>
@@ -22018,7 +22016,7 @@
         <v>-0.305492099924367</v>
       </c>
       <c r="R220" t="n">
-        <v>1.365</v>
+        <v>-0.0667152623401408</v>
       </c>
       <c r="S220" t="n">
         <v>-0.0340284869509766</v>
@@ -22113,7 +22111,7 @@
         <v>-0.151248964178053</v>
       </c>
       <c r="R221" t="n">
-        <v>-0.901</v>
+        <v>-0.0291206340418693</v>
       </c>
       <c r="S221" t="n">
         <v>-0.0223351143478937</v>
@@ -22208,7 +22206,7 @@
         <v>-0.0783999514670299</v>
       </c>
       <c r="R222" t="n">
-        <v>-0.901</v>
+        <v>-0.0280243179677463</v>
       </c>
       <c r="S222" t="n">
         <v>-0.0147733331045892</v>
@@ -22303,7 +22301,7 @@
         <v>-0.114631622173017</v>
       </c>
       <c r="R223" t="n">
-        <v>-0.901</v>
+        <v>-0.0267859547069128</v>
       </c>
       <c r="S223" t="n">
         <v>-0.0135099711225811</v>
@@ -22398,7 +22396,7 @@
         <v>-0.0901963250630905</v>
       </c>
       <c r="R224" t="n">
-        <v>-0.901</v>
+        <v>-0.0260833585584923</v>
       </c>
       <c r="S224" t="n">
         <v>-0.0136950413631103</v>
@@ -22493,7 +22491,7 @@
         <v>-0.0514955266221351</v>
       </c>
       <c r="R225" t="n">
-        <v>-2.15</v>
+        <v>-0.00390941256769256</v>
       </c>
       <c r="S225" t="n">
         <v>-0.0128565168020372</v>
@@ -22588,7 +22586,7 @@
         <v>-0.0186031784889458</v>
       </c>
       <c r="R226" t="n">
-        <v>0</v>
+        <v>-0.00267820231647668</v>
       </c>
       <c r="S226" t="n">
         <v>-0.014350571695556</v>
@@ -22683,7 +22681,7 @@
         <v>-0.0144964204239144</v>
       </c>
       <c r="R227" t="n">
-        <v>0</v>
+        <v>-0.00225053608046788</v>
       </c>
       <c r="S227" t="n">
         <v>-0.00988053397347205</v>
@@ -22778,7 +22776,7 @@
         <v>-0.013346169054578</v>
       </c>
       <c r="R228" t="n">
-        <v>0</v>
+        <v>-0.0028399763836967</v>
       </c>
       <c r="S228" t="n">
         <v>-0.00673794809319172</v>
@@ -22873,7 +22871,7 @@
         <v>-0.0113726885933712</v>
       </c>
       <c r="R229" t="n">
-        <v>0</v>
+        <v>-0.000298873614263938</v>
       </c>
       <c r="S229" t="n">
         <v>-0.00307865028129161</v>
@@ -22968,7 +22966,7 @@
         <v>-0.065543354191929</v>
       </c>
       <c r="R230" t="n">
-        <v>0</v>
+        <v>-0.000293409301204765</v>
       </c>
       <c r="S230" t="n">
         <v>-0.0013746041848217</v>
@@ -23063,7 +23061,7 @@
         <v>-0.0550751472029324</v>
       </c>
       <c r="R231" t="n">
-        <v>0</v>
+        <v>-0.000286664433782754</v>
       </c>
       <c r="S231" t="n">
         <v>-0.00103750585405049</v>
@@ -23158,7 +23156,7 @@
         <v>-0.0514266229727243</v>
       </c>
       <c r="R232" t="n">
-        <v>0</v>
+        <v>-0.000281037430917544</v>
       </c>
       <c r="S232" t="n">
         <v>-0.0010215825461172</v>
@@ -23253,7 +23251,7 @@
         <v>-0.0480629733680494</v>
       </c>
       <c r="R233" t="n">
-        <v>0</v>
+        <v>0.00020307512422245</v>
       </c>
       <c r="S233" t="n">
         <v>-0.00101704678480214</v>
@@ -23348,7 +23346,7 @@
         <v>-0.0420127997662854</v>
       </c>
       <c r="R234" t="n">
-        <v>0</v>
+        <v>0.00019938519262096</v>
       </c>
       <c r="S234" t="n">
         <v>-0.00102183495765849</v>
@@ -23443,7 +23441,7 @@
         <v>-0.0391679966473345</v>
       </c>
       <c r="R235" t="n">
-        <v>0</v>
+        <v>0.000195472164597558</v>
       </c>
       <c r="S235" t="n">
         <v>-0.000602817314630225</v>
@@ -23538,7 +23536,7 @@
         <v>-0.0383046594556231</v>
       </c>
       <c r="R236" t="n">
-        <v>0</v>
+        <v>0.00019200497056138</v>
       </c>
       <c r="S236" t="n">
         <v>-0.000601315167640283</v>
@@ -23633,7 +23631,7 @@
         <v>-0.038621710072626</v>
       </c>
       <c r="R237" t="n">
-        <v>0</v>
+        <v>0.000443326345424968</v>
       </c>
       <c r="S237" t="n">
         <v>-0.000601522800031365</v>

</xml_diff>

<commit_message>
fim results february 2025
</commit_message>
<xml_diff>
--- a/results/02-2025/beta/contributions-02-2025.xlsx
+++ b/results/02-2025/beta/contributions-02-2025.xlsx
@@ -21980,7 +21980,7 @@
         <v>0.0634323597791169</v>
       </c>
       <c r="F220" t="n">
-        <v>0.366579702932097</v>
+        <v>0.381138305063804</v>
       </c>
       <c r="G220" t="n">
         <v>-0.0396624458302889</v>
@@ -22043,19 +22043,19 @@
         <v>-0.150089202783916</v>
       </c>
       <c r="AA220" t="n">
-        <v>0.172717284908603</v>
+        <v>0.18730566625316</v>
       </c>
       <c r="AB220" t="n">
         <v>-0.1723691927932</v>
       </c>
       <c r="AC220" t="n">
-        <v>0.000660698686437814</v>
+        <v>0.0152754926875542</v>
       </c>
       <c r="AD220" t="n">
-        <v>0.486817256049722</v>
+        <v>0.501432050050839</v>
       </c>
       <c r="AE220" t="n">
-        <v>0.034580250253828</v>
+        <v>0.0382339487541071</v>
       </c>
     </row>
     <row r="221">
@@ -22069,88 +22069,88 @@
         <v>-1</v>
       </c>
       <c r="D221" t="n">
-        <v>0.0617366651178105</v>
+        <v>0.107150873316688</v>
       </c>
       <c r="E221" t="n">
-        <v>-0.0271804374498667</v>
+        <v>-0.011366028688026</v>
       </c>
       <c r="F221" t="n">
-        <v>0.321814767184305</v>
+        <v>0.352570134160248</v>
       </c>
       <c r="G221" t="n">
-        <v>-0.0115804452403324</v>
+        <v>-0.00616450493471536</v>
       </c>
       <c r="H221" t="n">
-        <v>-0.044015041837005</v>
+        <v>-0.043263388877005</v>
       </c>
       <c r="I221" t="n">
-        <v>-0.133713751969694</v>
+        <v>-0.134158072261678</v>
       </c>
       <c r="J221" t="n">
-        <v>0.0129282606856408</v>
+        <v>0.0132320470285215</v>
       </c>
       <c r="K221" t="n">
-        <v>0.181403623200494</v>
+        <v>0.173003157723465</v>
       </c>
       <c r="L221" t="n">
-        <v>0.0108224364660076</v>
+        <v>0.00964915074866303</v>
       </c>
       <c r="M221" t="n">
         <v>0</v>
       </c>
       <c r="N221" t="n">
-        <v>-0.100695753974172</v>
+        <v>-0.100852977945604</v>
       </c>
       <c r="O221" t="n">
-        <v>-0.000173348077153912</v>
+        <v>-0.000173512536473991</v>
       </c>
       <c r="P221" t="n">
-        <v>0.00378313170587277</v>
+        <v>0.00364483446927851</v>
       </c>
       <c r="Q221" t="n">
-        <v>-0.151248964178053</v>
+        <v>-0.151329872047867</v>
       </c>
       <c r="R221" t="n">
-        <v>-0.0291206340418693</v>
+        <v>-0.0291775594193379</v>
       </c>
       <c r="S221" t="n">
-        <v>-0.0223351143478937</v>
+        <v>-0.0223872422655659</v>
       </c>
       <c r="T221" t="n">
-        <v>-0.0266022706668706</v>
+        <v>-0.0266478280873095</v>
       </c>
       <c r="U221" t="n">
-        <v>-0.0307569738034392</v>
+        <v>-0.0308134352314298</v>
       </c>
       <c r="V221" t="n">
-        <v>-0.0000523223603890049</v>
+        <v>-0.0000541637421126199</v>
       </c>
       <c r="W221" t="n">
-        <v>0.159581805374586</v>
+        <v>0.152861670376723</v>
       </c>
       <c r="X221" t="n">
-        <v>0.14627477418583</v>
+        <v>0.145236653229646</v>
       </c>
       <c r="Y221" t="n">
-        <v>0.0227646706299541</v>
+        <v>0.0741955630503683</v>
       </c>
       <c r="Z221" t="n">
-        <v>0.0117915570379896</v>
+        <v>0.0215892815782934</v>
       </c>
       <c r="AA221" t="n">
-        <v>0.145965665101365</v>
+        <v>0.182792492079279</v>
       </c>
       <c r="AB221" t="n">
-        <v>0.14137792552272</v>
+        <v>0.123452917116291</v>
       </c>
       <c r="AC221" t="n">
-        <v>0.287129530360456</v>
+        <v>0.306011520747354</v>
       </c>
       <c r="AD221" t="n">
-        <v>0.3216857580284</v>
+        <v>0.401796365376016</v>
       </c>
       <c r="AE221" t="n">
-        <v>0.230851117463381</v>
+        <v>0.254532467800564</v>
       </c>
     </row>
     <row r="222">
@@ -22164,88 +22164,88 @@
         <v>0</v>
       </c>
       <c r="D222" t="n">
-        <v>-0.34807813640873</v>
+        <v>-0.34812269649394</v>
       </c>
       <c r="E222" t="n">
-        <v>-0.161620660751828</v>
+        <v>-0.161446108278581</v>
       </c>
       <c r="F222" t="n">
-        <v>-0.0414174105139845</v>
+        <v>0.0107685291377733</v>
       </c>
       <c r="G222" t="n">
-        <v>-0.0137899957628793</v>
+        <v>-0.00362511891593439</v>
       </c>
       <c r="H222" t="n">
-        <v>-0.0403999871395128</v>
+        <v>-0.0386102743233363</v>
       </c>
       <c r="I222" t="n">
-        <v>0.027955186001023</v>
+        <v>0.0272327215780774</v>
       </c>
       <c r="J222" t="n">
-        <v>0.0133818767419251</v>
+        <v>0.0140214378438707</v>
       </c>
       <c r="K222" t="n">
-        <v>0.0326908480679156</v>
+        <v>0.0104374406536559</v>
       </c>
       <c r="L222" t="n">
-        <v>0.0305593768089365</v>
+        <v>0.0286274791953285</v>
       </c>
       <c r="M222" t="n">
         <v>0</v>
       </c>
       <c r="N222" t="n">
-        <v>-0.0969196410703134</v>
+        <v>-0.0969948095236936</v>
       </c>
       <c r="O222" t="n">
         <v>0</v>
       </c>
       <c r="P222" t="n">
-        <v>-0.000557558363155953</v>
+        <v>-0.000872664091383299</v>
       </c>
       <c r="Q222" t="n">
-        <v>-0.0783999514670299</v>
+        <v>-0.0787045902525759</v>
       </c>
       <c r="R222" t="n">
-        <v>-0.0280243179677463</v>
+        <v>-0.0280715359290164</v>
       </c>
       <c r="S222" t="n">
-        <v>-0.0147733331045892</v>
+        <v>-0.0148326651704783</v>
       </c>
       <c r="T222" t="n">
-        <v>-0.010488174256784</v>
+        <v>-0.010526635232305</v>
       </c>
       <c r="U222" t="n">
-        <v>-0.0300407786324789</v>
+        <v>-0.03008222459157</v>
       </c>
       <c r="V222" t="n">
-        <v>-0.000769388632245321</v>
+        <v>-0.000772880260457906</v>
       </c>
       <c r="W222" t="n">
-        <v>0.205529202507233</v>
+        <v>0.247727825279121</v>
       </c>
       <c r="X222" t="n">
-        <v>0.0209331710080876</v>
+        <v>0.0449923871213833</v>
       </c>
       <c r="Y222" t="n">
-        <v>-0.671876217810323</v>
+        <v>-0.671715703854223</v>
       </c>
       <c r="Z222" t="n">
-        <v>0.162177420649765</v>
+        <v>0.162146899081702</v>
       </c>
       <c r="AA222" t="n">
-        <v>-0.0542621439539953</v>
+        <v>0.00980026746305165</v>
       </c>
       <c r="AB222" t="n">
-        <v>0.0300628414863404</v>
+        <v>0.0713327295060325</v>
       </c>
       <c r="AC222" t="n">
-        <v>-0.0241821186160988</v>
+        <v>0.0811256283481254</v>
       </c>
       <c r="AD222" t="n">
-        <v>-0.533880915776657</v>
+        <v>-0.428443176424396</v>
       </c>
       <c r="AE222" t="n">
-        <v>0.0986795733882548</v>
+        <v>0.148720358563503</v>
       </c>
     </row>
     <row r="223">
@@ -22259,88 +22259,88 @@
         <v>0</v>
       </c>
       <c r="D223" t="n">
-        <v>-0.247817697871643</v>
+        <v>-0.247897737351378</v>
       </c>
       <c r="E223" t="n">
-        <v>-0.198483961223232</v>
+        <v>-0.198269595892895</v>
       </c>
       <c r="F223" t="n">
-        <v>-0.0135610884496303</v>
+        <v>0.0191635970233239</v>
       </c>
       <c r="G223" t="n">
-        <v>-0.0210546720250031</v>
+        <v>-0.0197427348749497</v>
       </c>
       <c r="H223" t="n">
-        <v>-0.0302241829692944</v>
+        <v>-0.029584098165249</v>
       </c>
       <c r="I223" t="n">
-        <v>0.187449897075292</v>
+        <v>0.18707964577705</v>
       </c>
       <c r="J223" t="n">
-        <v>0.0071406981663046</v>
+        <v>0.00735737740620022</v>
       </c>
       <c r="K223" t="n">
-        <v>-0.0233939417202723</v>
+        <v>-0.0330876535616735</v>
       </c>
       <c r="L223" t="n">
-        <v>0.0293258259415457</v>
+        <v>0.0286394445162739</v>
       </c>
       <c r="M223" t="n">
         <v>0</v>
       </c>
       <c r="N223" t="n">
-        <v>-0.09511751915457</v>
+        <v>-0.0950805508069859</v>
       </c>
       <c r="O223" t="n">
         <v>0</v>
       </c>
       <c r="P223" t="n">
-        <v>-0.00206150910572198</v>
+        <v>-0.00216932574867619</v>
       </c>
       <c r="Q223" t="n">
-        <v>-0.114631622173017</v>
+        <v>-0.11449131433406</v>
       </c>
       <c r="R223" t="n">
-        <v>-0.0267859547069128</v>
+        <v>-0.0267845543866995</v>
       </c>
       <c r="S223" t="n">
-        <v>-0.0135099711225811</v>
+        <v>-0.0135215529242429</v>
       </c>
       <c r="T223" t="n">
-        <v>-0.0100402353603435</v>
+        <v>-0.0100469027546833</v>
       </c>
       <c r="U223" t="n">
-        <v>-0.0237813599967932</v>
+        <v>-0.0237798353383869</v>
       </c>
       <c r="V223" t="n">
-        <v>-0.00144773838632898</v>
+        <v>-0.0014480049834142</v>
       </c>
       <c r="W223" t="n">
-        <v>0.202869926127886</v>
+        <v>0.255069401121969</v>
       </c>
       <c r="X223" t="n">
-        <v>0.00723031025459963</v>
+        <v>0.0330444313257097</v>
       </c>
       <c r="Y223" t="n">
-        <v>-0.451121359028853</v>
+        <v>-0.451072062860655</v>
       </c>
       <c r="Z223" t="n">
-        <v>0.00481969993397691</v>
+        <v>0.00490472961638176</v>
       </c>
       <c r="AA223" t="n">
-        <v>0.129855075427962</v>
+        <v>0.164324700557513</v>
       </c>
       <c r="AB223" t="n">
-        <v>-0.0710217224021438</v>
+        <v>-0.00317405570746418</v>
       </c>
       <c r="AC223" t="n">
-        <v>0.0589301400176166</v>
+        <v>0.161156121911072</v>
       </c>
       <c r="AD223" t="n">
-        <v>-0.387371519077259</v>
+        <v>-0.285011211333202</v>
       </c>
       <c r="AE223" t="n">
-        <v>-0.0281873551939488</v>
+        <v>0.0474435069173137</v>
       </c>
     </row>
     <row r="224">
@@ -22354,88 +22354,88 @@
         <v>0</v>
       </c>
       <c r="D224" t="n">
-        <v>-0.165495035219233</v>
+        <v>-0.165623756991551</v>
       </c>
       <c r="E224" t="n">
-        <v>-0.187086954711526</v>
+        <v>-0.186884898300513</v>
       </c>
       <c r="F224" t="n">
-        <v>0.0396444150512974</v>
+        <v>0.0635512501973908</v>
       </c>
       <c r="G224" t="n">
-        <v>-0.0205054423792219</v>
+        <v>-0.0180879943783451</v>
       </c>
       <c r="H224" t="n">
-        <v>-0.0442496312877029</v>
+        <v>-0.0436583349794452</v>
       </c>
       <c r="I224" t="n">
-        <v>0.186248923662574</v>
+        <v>0.18586463155258</v>
       </c>
       <c r="J224" t="n">
-        <v>0.00758182161221361</v>
+        <v>0.00777369979516931</v>
       </c>
       <c r="K224" t="n">
-        <v>-0.0540510765691226</v>
+        <v>-0.0629538330084869</v>
       </c>
       <c r="L224" t="n">
-        <v>0.0101245174506297</v>
+        <v>0.00951346206366038</v>
       </c>
       <c r="M224" t="n">
         <v>0</v>
       </c>
       <c r="N224" t="n">
-        <v>-0.000996291238913357</v>
+        <v>-0.000996294750735312</v>
       </c>
       <c r="O224" t="n">
         <v>0</v>
       </c>
       <c r="P224" t="n">
-        <v>-0.00383432122119921</v>
+        <v>-0.00392923037084015</v>
       </c>
       <c r="Q224" t="n">
-        <v>-0.0901963250630905</v>
+        <v>-0.0900478608909075</v>
       </c>
       <c r="R224" t="n">
-        <v>-0.0260833585584923</v>
+        <v>-0.0260749383790248</v>
       </c>
       <c r="S224" t="n">
-        <v>-0.0136950413631103</v>
+        <v>-0.013701462629103</v>
       </c>
       <c r="T224" t="n">
-        <v>-0.00846909867248599</v>
+        <v>-0.00847322450313509</v>
       </c>
       <c r="U224" t="n">
-        <v>0.000187488384394089</v>
+        <v>0.000180292621668077</v>
       </c>
       <c r="V224" t="n">
-        <v>-0.000422393250818566</v>
+        <v>-0.000422876186853873</v>
       </c>
       <c r="W224" t="n">
-        <v>0.17739808102058</v>
+        <v>0.229874822529572</v>
       </c>
       <c r="X224" t="n">
-        <v>0.0394457475386531</v>
+        <v>0.0650628541464284</v>
       </c>
       <c r="Y224" t="n">
-        <v>-0.21962636599384</v>
+        <v>-0.219720493872276</v>
       </c>
       <c r="Z224" t="n">
-        <v>-0.132955623936919</v>
+        <v>-0.132788161419787</v>
       </c>
       <c r="AA224" t="n">
-        <v>0.168774044148235</v>
+        <v>0.195457333484598</v>
       </c>
       <c r="AB224" t="n">
-        <v>0.0296417062074377</v>
+        <v>0.0983516726802031</v>
       </c>
       <c r="AC224" t="n">
-        <v>0.198362932650413</v>
+        <v>0.29360592812621</v>
       </c>
       <c r="AD224" t="n">
-        <v>-0.154219057280346</v>
+        <v>-0.0589027271658538</v>
       </c>
       <c r="AE224" t="n">
-        <v>-0.188446433526466</v>
+        <v>-0.0926401873868594</v>
       </c>
     </row>
     <row r="225">
@@ -22449,88 +22449,88 @@
         <v>0</v>
       </c>
       <c r="D225" t="n">
-        <v>-0.1633236700508</v>
+        <v>-0.16345070293878</v>
       </c>
       <c r="E225" t="n">
-        <v>-0.186117706256797</v>
+        <v>-0.185916696647066</v>
       </c>
       <c r="F225" t="n">
-        <v>0.0540647382829215</v>
+        <v>0.0776712627364136</v>
       </c>
       <c r="G225" t="n">
-        <v>-0.0119604342470875</v>
+        <v>-0.00951916342499131</v>
       </c>
       <c r="H225" t="n">
-        <v>-0.0392809380894438</v>
+        <v>-0.0386834152565656</v>
       </c>
       <c r="I225" t="n">
-        <v>0.0731387415431299</v>
+        <v>0.0727857675446842</v>
       </c>
       <c r="J225" t="n">
-        <v>0.00895726853744521</v>
+        <v>0.00914651764625598</v>
       </c>
       <c r="K225" t="n">
-        <v>-0.143662853717726</v>
+        <v>-0.152434624461755</v>
       </c>
       <c r="L225" t="n">
-        <v>0.0313941553807056</v>
+        <v>0.031069649235347</v>
       </c>
       <c r="M225" t="n">
         <v>0</v>
       </c>
       <c r="N225" t="n">
-        <v>-0.000974759284971623</v>
+        <v>-0.000974558269637336</v>
       </c>
       <c r="O225" t="n">
         <v>0</v>
       </c>
       <c r="P225" t="n">
-        <v>-0.00477537274558585</v>
+        <v>-0.00486879867638218</v>
       </c>
       <c r="Q225" t="n">
-        <v>-0.0514955266221351</v>
+        <v>-0.0513879347388036</v>
       </c>
       <c r="R225" t="n">
-        <v>-0.00390941256769256</v>
+        <v>-0.00390945658319908</v>
       </c>
       <c r="S225" t="n">
-        <v>-0.0128565168020372</v>
+        <v>-0.0128604703583512</v>
       </c>
       <c r="T225" t="n">
-        <v>-0.00767421630840517</v>
+        <v>-0.0076769927369462</v>
       </c>
       <c r="U225" t="n">
-        <v>0.000127213238151998</v>
+        <v>0.000120018142809031</v>
       </c>
       <c r="V225" t="n">
-        <v>-0.000392391910669682</v>
+        <v>-0.0003928012630834</v>
       </c>
       <c r="W225" t="n">
-        <v>0.124381472679477</v>
+        <v>0.176375078029272</v>
       </c>
       <c r="X225" t="n">
-        <v>0.0202073513158241</v>
+        <v>0.0456891245892075</v>
       </c>
       <c r="Y225" t="n">
-        <v>-0.269854040412236</v>
+        <v>-0.269913096075334</v>
       </c>
       <c r="Z225" t="n">
-        <v>-0.0795873358953607</v>
+        <v>-0.0794543035105125</v>
       </c>
       <c r="AA225" t="n">
-        <v>0.0849343034815282</v>
+        <v>0.111404066224449</v>
       </c>
       <c r="AB225" t="n">
-        <v>-0.0494301430044199</v>
+        <v>0.0190653212280896</v>
       </c>
       <c r="AC225" t="n">
-        <v>0.035548552201779</v>
+        <v>0.130446916034948</v>
       </c>
       <c r="AD225" t="n">
-        <v>-0.313892824105818</v>
+        <v>-0.218920483550899</v>
       </c>
       <c r="AE225" t="n">
-        <v>-0.34734107906002</v>
+        <v>-0.247819399618588</v>
       </c>
     </row>
     <row r="226">
@@ -22544,88 +22544,88 @@
         <v>0</v>
       </c>
       <c r="D226" t="n">
-        <v>-0.145518641391626</v>
+        <v>-0.145631825556942</v>
       </c>
       <c r="E226" t="n">
-        <v>-0.184944137503267</v>
+        <v>-0.184744395363472</v>
       </c>
       <c r="F226" t="n">
-        <v>-0.0329407638178037</v>
+        <v>-0.00867677039099331</v>
       </c>
       <c r="G226" t="n">
-        <v>-0.0173683379726714</v>
+        <v>-0.0148987391943528</v>
       </c>
       <c r="H226" t="n">
-        <v>-0.024866739985262</v>
+        <v>-0.0242704833921742</v>
       </c>
       <c r="I226" t="n">
-        <v>0.316216081744669</v>
+        <v>0.315692954023002</v>
       </c>
       <c r="J226" t="n">
-        <v>0.00707160729974725</v>
+        <v>0.00725991836711011</v>
       </c>
       <c r="K226" t="n">
-        <v>-0.134207262920954</v>
+        <v>-0.150055021092008</v>
       </c>
       <c r="L226" t="n">
-        <v>0.0106764229020771</v>
+        <v>0.010053390320148</v>
       </c>
       <c r="M226" t="n">
         <v>0</v>
       </c>
       <c r="N226" t="n">
-        <v>-0.000952400669173704</v>
+        <v>-0.000952000380025069</v>
       </c>
       <c r="O226" t="n">
         <v>0</v>
       </c>
       <c r="P226" t="n">
-        <v>-0.00432536131802174</v>
+        <v>-0.00441793686412618</v>
       </c>
       <c r="Q226" t="n">
-        <v>-0.0186031784889458</v>
+        <v>-0.018510124049966</v>
       </c>
       <c r="R226" t="n">
-        <v>-0.00267820231647668</v>
+        <v>-0.00267817606184217</v>
       </c>
       <c r="S226" t="n">
-        <v>-0.014350571695556</v>
+        <v>-0.0143507467896208</v>
       </c>
       <c r="T226" t="n">
-        <v>-0.00706636199314988</v>
+        <v>-0.00706784131765174</v>
       </c>
       <c r="U226" t="n">
-        <v>-0.000157298916468364</v>
+        <v>-0.000164333077580123</v>
       </c>
       <c r="V226" t="n">
-        <v>-0.000341473817191051</v>
+        <v>-0.000341829275316612</v>
       </c>
       <c r="W226" t="n">
-        <v>0.0979129185916273</v>
+        <v>0.0944351457288708</v>
       </c>
       <c r="X226" t="n">
-        <v>0.0237885321257464</v>
+        <v>0.0235824536144519</v>
       </c>
       <c r="Y226" t="n">
-        <v>-0.199178787505235</v>
+        <v>-0.19925767927302</v>
       </c>
       <c r="Z226" t="n">
-        <v>-0.131283991389658</v>
+        <v>-0.131118541647394</v>
       </c>
       <c r="AA226" t="n">
-        <v>0.24832683879382</v>
+        <v>0.275239234378854</v>
       </c>
       <c r="AB226" t="n">
-        <v>-0.0501642591803662</v>
+        <v>-0.0703196787891154</v>
       </c>
       <c r="AC226" t="n">
-        <v>0.198294829060836</v>
+        <v>0.205125122840537</v>
       </c>
       <c r="AD226" t="n">
-        <v>-0.132167949834057</v>
+        <v>-0.125251098079876</v>
       </c>
       <c r="AE226" t="n">
-        <v>-0.24691283757437</v>
+        <v>-0.172021380032458</v>
       </c>
     </row>
     <row r="227">
@@ -22639,31 +22639,31 @@
         <v>0</v>
       </c>
       <c r="D227" t="n">
-        <v>-0.147252579330539</v>
+        <v>-0.147367112149997</v>
       </c>
       <c r="E227" t="n">
-        <v>-0.195925771034664</v>
+        <v>-0.195714168583914</v>
       </c>
       <c r="F227" t="n">
-        <v>-0.0492959498885515</v>
+        <v>-0.0332189410306446</v>
       </c>
       <c r="G227" t="n">
-        <v>-0.00133507438583787</v>
+        <v>-0.00332478686040428</v>
       </c>
       <c r="H227" t="n">
-        <v>-0.0250034593378032</v>
+        <v>-0.0249874737051534</v>
       </c>
       <c r="I227" t="n">
-        <v>0.250585098634257</v>
+        <v>0.250424968075351</v>
       </c>
       <c r="J227" t="n">
-        <v>0.00843894731196212</v>
+        <v>0.00843355229919704</v>
       </c>
       <c r="K227" t="n">
-        <v>-0.134388545936565</v>
+        <v>-0.144165636180601</v>
       </c>
       <c r="L227" t="n">
-        <v>0.011015700007863</v>
+        <v>0.0110086577109504</v>
       </c>
       <c r="M227" t="n">
         <v>0</v>
@@ -22675,52 +22675,52 @@
         <v>0</v>
       </c>
       <c r="P227" t="n">
-        <v>-0.0041481801555767</v>
+        <v>-0.00414552816847914</v>
       </c>
       <c r="Q227" t="n">
-        <v>-0.0144964204239144</v>
+        <v>-0.0142818564061106</v>
       </c>
       <c r="R227" t="n">
-        <v>-0.00225053608046788</v>
+        <v>-0.0022490972874036</v>
       </c>
       <c r="S227" t="n">
-        <v>-0.00988053397347205</v>
+        <v>-0.0098742171520722</v>
       </c>
       <c r="T227" t="n">
-        <v>-0.00649469655903006</v>
+        <v>-0.00649054439537933</v>
       </c>
       <c r="U227" t="n">
-        <v>-0.000192893823749738</v>
+        <v>-0.000192770505025867</v>
       </c>
       <c r="V227" t="n">
-        <v>-0.000335201400242419</v>
+        <v>-0.000334987103008061</v>
       </c>
       <c r="W227" t="n">
-        <v>0.0970894928520597</v>
+        <v>0.0982709301114543</v>
       </c>
       <c r="X227" t="n">
-        <v>0.0185822211160797</v>
+        <v>0.0190887418329028</v>
       </c>
       <c r="Y227" t="n">
-        <v>-0.233470525752245</v>
+        <v>-0.233530005341908</v>
       </c>
       <c r="Z227" t="n">
-        <v>-0.109707824612958</v>
+        <v>-0.109551275392002</v>
       </c>
       <c r="AA227" t="n">
-        <v>0.183560777113104</v>
+        <v>0.197463041084425</v>
       </c>
       <c r="AB227" t="n">
-        <v>-0.0453604341099568</v>
+        <v>-0.0532154834629245</v>
       </c>
       <c r="AC227" t="n">
-        <v>0.138288625023113</v>
+        <v>0.144359020251566</v>
       </c>
       <c r="AD227" t="n">
-        <v>-0.20488972534209</v>
+        <v>-0.198722260482345</v>
       </c>
       <c r="AE227" t="n">
-        <v>-0.201292389140578</v>
+        <v>-0.150449142319744</v>
       </c>
     </row>
     <row r="228">
@@ -22734,31 +22734,31 @@
         <v>0</v>
       </c>
       <c r="D228" t="n">
-        <v>-0.139582711339068</v>
+        <v>-0.139691278547532</v>
       </c>
       <c r="E228" t="n">
-        <v>-0.185812886698803</v>
+        <v>-0.185612206298268</v>
       </c>
       <c r="F228" t="n">
-        <v>0.0321916200794655</v>
+        <v>0.0408990275306336</v>
       </c>
       <c r="G228" t="n">
-        <v>0.0126215919672404</v>
+        <v>0.0106520855188045</v>
       </c>
       <c r="H228" t="n">
-        <v>-0.0130502913407651</v>
+        <v>-0.0130419479830668</v>
       </c>
       <c r="I228" t="n">
-        <v>0.0774548003327265</v>
+        <v>0.077405289584621</v>
       </c>
       <c r="J228" t="n">
-        <v>0.009871610726193</v>
+        <v>0.00986529982926714</v>
       </c>
       <c r="K228" t="n">
-        <v>-0.129678398898587</v>
+        <v>-0.139223319797929</v>
       </c>
       <c r="L228" t="n">
-        <v>0.0111976073278526</v>
+        <v>0.0111904487412982</v>
       </c>
       <c r="M228" t="n">
         <v>0</v>
@@ -22770,52 +22770,52 @@
         <v>0</v>
       </c>
       <c r="P228" t="n">
-        <v>-0.00454026460507237</v>
+        <v>-0.00453736195097931</v>
       </c>
       <c r="Q228" t="n">
-        <v>-0.013346169054578</v>
+        <v>-0.0131372879719407</v>
       </c>
       <c r="R228" t="n">
-        <v>-0.0028399763836967</v>
+        <v>-0.00283816075296156</v>
       </c>
       <c r="S228" t="n">
-        <v>-0.00673794809319172</v>
+        <v>-0.00673364041288035</v>
       </c>
       <c r="T228" t="n">
-        <v>-0.00579336891339557</v>
+        <v>-0.00578966512410781</v>
       </c>
       <c r="U228" t="n">
-        <v>-0.00730033596154624</v>
+        <v>-0.00729566873282012</v>
       </c>
       <c r="V228" t="n">
-        <v>-0.000327381757716453</v>
+        <v>-0.000327172459639406</v>
       </c>
       <c r="W228" t="n">
-        <v>0.091675900887246</v>
+        <v>0.0924703218328053</v>
       </c>
       <c r="X228" t="n">
-        <v>0.0163594046580318</v>
+        <v>0.0168053403300093</v>
       </c>
       <c r="Y228" t="n">
-        <v>-0.175140787664719</v>
+        <v>-0.175226623214915</v>
       </c>
       <c r="Z228" t="n">
-        <v>-0.150254810373152</v>
+        <v>-0.150076861630886</v>
       </c>
       <c r="AA228" t="n">
-        <v>0.119053518235001</v>
+        <v>0.125738296130897</v>
       </c>
       <c r="AB228" t="n">
-        <v>-0.051206665140721</v>
+        <v>-0.0592821129504645</v>
       </c>
       <c r="AC228" t="n">
-        <v>0.0679118308361764</v>
+        <v>0.0665356657064532</v>
       </c>
       <c r="AD228" t="n">
-        <v>-0.257483767201695</v>
+        <v>-0.258767819139347</v>
       </c>
       <c r="AE228" t="n">
-        <v>-0.227108566620915</v>
+        <v>-0.200415415313117</v>
       </c>
     </row>
     <row r="229">
@@ -22829,31 +22829,31 @@
         <v>0</v>
       </c>
       <c r="D229" t="n">
-        <v>-0.157724716309526</v>
+        <v>-0.157847394340289</v>
       </c>
       <c r="E229" t="n">
-        <v>-0.196517525634564</v>
+        <v>-0.196305284080939</v>
       </c>
       <c r="F229" t="n">
-        <v>0.0560394532463033</v>
+        <v>0.0626635817444789</v>
       </c>
       <c r="G229" t="n">
-        <v>0.0242147879382389</v>
+        <v>0.0227170465156699</v>
       </c>
       <c r="H229" t="n">
-        <v>-0.00556296467863358</v>
+        <v>-0.00555940819187405</v>
       </c>
       <c r="I229" t="n">
-        <v>-0.0529830647677751</v>
+        <v>-0.0529491890680316</v>
       </c>
       <c r="J229" t="n">
-        <v>0.0101324537434585</v>
+        <v>0.0101259760929233</v>
       </c>
       <c r="K229" t="n">
-        <v>-0.0799047434898798</v>
+        <v>-0.0893103752649634</v>
       </c>
       <c r="L229" t="n">
-        <v>0.0113318021334119</v>
+        <v>0.0113245577579837</v>
       </c>
       <c r="M229" t="n">
         <v>0</v>
@@ -22865,52 +22865,52 @@
         <v>0</v>
       </c>
       <c r="P229" t="n">
-        <v>-0.00465924195506322</v>
+        <v>-0.00465626323656946</v>
       </c>
       <c r="Q229" t="n">
-        <v>-0.0113726885933712</v>
+        <v>-0.0112121827482052</v>
       </c>
       <c r="R229" t="n">
-        <v>-0.000298873614263938</v>
+        <v>-0.000298682541668834</v>
       </c>
       <c r="S229" t="n">
-        <v>-0.00307865028129161</v>
+        <v>-0.00307668206262129</v>
       </c>
       <c r="T229" t="n">
-        <v>-0.00322024472586091</v>
+        <v>-0.00321818598360054</v>
       </c>
       <c r="U229" t="n">
-        <v>-0.00616989762216411</v>
+        <v>-0.0061659531098135</v>
       </c>
       <c r="V229" t="n">
-        <v>-0.000322025182466009</v>
+        <v>-0.000321819308917466</v>
       </c>
       <c r="W229" t="n">
-        <v>0.0954632874642013</v>
+        <v>0.0963273722433284</v>
       </c>
       <c r="X229" t="n">
-        <v>0.0150333400316784</v>
+        <v>0.0154431320489032</v>
       </c>
       <c r="Y229" t="n">
-        <v>-0.21823771920789</v>
+        <v>-0.218321730117281</v>
       </c>
       <c r="Z229" t="n">
-        <v>-0.1360045227362</v>
+        <v>-0.135830948303947</v>
       </c>
       <c r="AA229" t="n">
-        <v>0.0318707078616372</v>
+        <v>0.0370299617194311</v>
       </c>
       <c r="AB229" t="n">
-        <v>0.0128865712822585</v>
+        <v>0.00492959763518629</v>
       </c>
       <c r="AC229" t="n">
-        <v>0.0447529126725451</v>
+        <v>0.0419576177996649</v>
       </c>
       <c r="AD229" t="n">
-        <v>-0.309489329271545</v>
+        <v>-0.312195060621563</v>
       </c>
       <c r="AE229" t="n">
-        <v>-0.226007692912347</v>
+        <v>-0.223734059580783</v>
       </c>
     </row>
     <row r="230">
@@ -22924,31 +22924,31 @@
         <v>0</v>
       </c>
       <c r="D230" t="n">
-        <v>-6.26479453431126</v>
+        <v>-6.26966728142779</v>
       </c>
       <c r="E230" t="n">
-        <v>-10.8560172782225</v>
+        <v>-10.8442926345</v>
       </c>
       <c r="F230" t="n">
-        <v>7.3454506290301</v>
+        <v>7.30983911401378</v>
       </c>
       <c r="G230" t="n">
-        <v>4.12951775549395</v>
+        <v>4.13093177963875</v>
       </c>
       <c r="H230" t="n">
-        <v>0.224607894671299</v>
+        <v>0.224464357740274</v>
       </c>
       <c r="I230" t="n">
-        <v>-2.09966831049962</v>
+        <v>-2.09832107244378</v>
       </c>
       <c r="J230" t="n">
-        <v>0.0815859936955833</v>
+        <v>0.0815338425525267</v>
       </c>
       <c r="K230" t="n">
-        <v>-7.06295883538682</v>
+        <v>-7.04416989103243</v>
       </c>
       <c r="L230" t="n">
-        <v>-0.729227778327072</v>
+        <v>-0.728760980647201</v>
       </c>
       <c r="M230" t="n">
         <v>0</v>
@@ -22960,52 +22960,52 @@
         <v>0</v>
       </c>
       <c r="P230" t="n">
-        <v>-0.0958835724542424</v>
+        <v>-0.0958222629062048</v>
       </c>
       <c r="Q230" t="n">
-        <v>-0.065543354191929</v>
+        <v>-0.0656680179440577</v>
       </c>
       <c r="R230" t="n">
-        <v>-0.000293409301204765</v>
+        <v>-0.000293221721984725</v>
       </c>
       <c r="S230" t="n">
-        <v>-0.0013746041848217</v>
+        <v>-0.0013737253862283</v>
       </c>
       <c r="T230" t="n">
-        <v>-0.00182087934196328</v>
+        <v>-0.00181971523414214</v>
       </c>
       <c r="U230" t="n">
-        <v>-0.00572334943650009</v>
+        <v>-0.00571969041232334</v>
       </c>
       <c r="V230" t="n">
-        <v>-0.000255678670957171</v>
+        <v>-0.000255515213330649</v>
       </c>
       <c r="W230" t="n">
-        <v>-5.95953831389001</v>
+        <v>-6.01889610366008</v>
       </c>
       <c r="X230" t="n">
-        <v>-0.989202006055241</v>
+        <v>-1.0163157276317</v>
       </c>
       <c r="Y230" t="n">
-        <v>-7.95065978167497</v>
+        <v>-7.95445474040605</v>
       </c>
       <c r="Z230" t="n">
-        <v>-9.17015203085884</v>
+        <v>-9.15950517552169</v>
       </c>
       <c r="AA230" t="n">
-        <v>9.57460158080813</v>
+        <v>9.5422179733159</v>
       </c>
       <c r="AB230" t="n">
-        <v>-15.624039272464</v>
+        <v>-15.6996103105912</v>
       </c>
       <c r="AC230" t="n">
-        <v>-4.47257206394178</v>
+        <v>-4.57786837434647</v>
       </c>
       <c r="AD230" t="n">
-        <v>-21.5933838764756</v>
+        <v>-21.6918282902742</v>
       </c>
       <c r="AE230" t="n">
-        <v>-5.59131167457273</v>
+        <v>-5.61537835762937</v>
       </c>
     </row>
     <row r="231">
@@ -23025,25 +23025,25 @@
         <v>#NUM!</v>
       </c>
       <c r="F231" t="n">
-        <v>7.22326359141172</v>
+        <v>7.1882316620937</v>
       </c>
       <c r="G231" t="n">
-        <v>4.07822811552373</v>
+        <v>4.07962742075285</v>
       </c>
       <c r="H231" t="n">
-        <v>0.233642378348238</v>
+        <v>0.233493070534625</v>
       </c>
       <c r="I231" t="n">
         <v>0</v>
       </c>
       <c r="J231" t="n">
-        <v>0.077048626303182</v>
+        <v>0.076999375157603</v>
       </c>
       <c r="K231" t="n">
-        <v>-6.91549834477872</v>
+        <v>-6.89714563482358</v>
       </c>
       <c r="L231" t="n">
-        <v>-0.722674889662615</v>
+        <v>-0.722212289365687</v>
       </c>
       <c r="M231" t="n">
         <v>0</v>
@@ -23055,31 +23055,31 @@
         <v>0</v>
       </c>
       <c r="P231" t="n">
-        <v>-0.0801402465448341</v>
+        <v>-0.0800890049273614</v>
       </c>
       <c r="Q231" t="n">
-        <v>-0.0550751472029324</v>
+        <v>-0.0551600601107615</v>
       </c>
       <c r="R231" t="n">
-        <v>-0.000286664433782754</v>
+        <v>-0.000286481166607188</v>
       </c>
       <c r="S231" t="n">
-        <v>-0.00103750585405049</v>
+        <v>-0.00103684256620762</v>
       </c>
       <c r="T231" t="n">
-        <v>-0.00153139088975758</v>
+        <v>-0.00153041185551572</v>
       </c>
       <c r="U231" t="n">
-        <v>-0.00526417013744741</v>
+        <v>-0.00526080467610503</v>
       </c>
       <c r="V231" t="n">
-        <v>-0.000249857728596157</v>
+        <v>-0.000249697992269249</v>
       </c>
       <c r="W231" t="n">
-        <v>-5.90663142049843</v>
+        <v>-5.96544292040139</v>
       </c>
       <c r="X231" t="n">
-        <v>-0.979949656153008</v>
+        <v>-1.00680905377357</v>
       </c>
       <c r="Y231" t="e">
         <v>#NUM!</v>
@@ -23088,19 +23088,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA231" t="n">
-        <v>11.2542730755514</v>
+        <v>11.2218875944419</v>
       </c>
       <c r="AB231" t="n">
-        <v>-15.360028117463</v>
+        <v>-15.4350124681937</v>
       </c>
       <c r="AC231" t="n">
-        <v>-2.2683924299434</v>
+        <v>-2.37164822706985</v>
       </c>
       <c r="AD231" t="n">
         <v>0</v>
       </c>
       <c r="AE231" t="n">
-        <v>-5.54008924323721</v>
+        <v>-5.56569779250878</v>
       </c>
     </row>
     <row r="232">
@@ -23120,25 +23120,25 @@
         <v>#NUM!</v>
       </c>
       <c r="F232" t="n">
-        <v>3.64373438602309</v>
+        <v>3.62575606280684</v>
       </c>
       <c r="G232" t="n">
-        <v>2.04738594373588</v>
+        <v>2.04810358325155</v>
       </c>
       <c r="H232" t="n">
-        <v>0.229091013713898</v>
+        <v>0.228944613301555</v>
       </c>
       <c r="I232" t="n">
         <v>0</v>
       </c>
       <c r="J232" t="n">
-        <v>0.0750005676272856</v>
+        <v>0.0749526254776213</v>
       </c>
       <c r="K232" t="n">
-        <v>-6.80044767472991</v>
+        <v>-6.78245317791429</v>
       </c>
       <c r="L232" t="n">
-        <v>-0.718815565347421</v>
+        <v>-0.718355438015802</v>
       </c>
       <c r="M232" t="n">
         <v>0</v>
@@ -23150,31 +23150,31 @@
         <v>0</v>
       </c>
       <c r="P232" t="n">
-        <v>-0.0741154535013819</v>
+        <v>-0.0740680646305141</v>
       </c>
       <c r="Q232" t="n">
-        <v>-0.0514266229727243</v>
+        <v>-0.0514975261317439</v>
       </c>
       <c r="R232" t="n">
-        <v>-0.000281037430917544</v>
+        <v>-0.0002808577611383</v>
       </c>
       <c r="S232" t="n">
-        <v>-0.0010215825461172</v>
+        <v>-0.00102092943827411</v>
       </c>
       <c r="T232" t="n">
-        <v>-0.00126584141024643</v>
+        <v>-0.00126503214492442</v>
       </c>
       <c r="U232" t="n">
-        <v>-0.00313374797706426</v>
+        <v>-0.00313174453349087</v>
       </c>
       <c r="V232" t="n">
-        <v>-0.000245035678081935</v>
+        <v>-0.000244879024604515</v>
       </c>
       <c r="W232" t="n">
-        <v>-5.87587580912618</v>
+        <v>-5.93436378271134</v>
       </c>
       <c r="X232" t="n">
-        <v>-0.974270252984039</v>
+        <v>-1.00097329776254</v>
       </c>
       <c r="Y232" t="e">
         <v>#NUM!</v>
@@ -23183,19 +23183,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA232" t="n">
-        <v>5.89619632942462</v>
+        <v>5.87913812367661</v>
       </c>
       <c r="AB232" t="n">
-        <v>-15.177865665081</v>
+        <v>-15.2525791973898</v>
       </c>
       <c r="AC232" t="n">
-        <v>-8.33965718153024</v>
+        <v>-8.42927053661975</v>
       </c>
       <c r="AD232" t="n">
         <v>0</v>
       </c>
       <c r="AE232" t="n">
-        <v>-5.47571830143678</v>
+        <v>-5.50100583772395</v>
       </c>
     </row>
     <row r="233">
@@ -23215,25 +23215,25 @@
         <v>#NUM!</v>
       </c>
       <c r="F233" t="n">
-        <v>3.59826206375921</v>
+        <v>3.58050010044361</v>
       </c>
       <c r="G233" t="n">
-        <v>2.03142347423668</v>
+        <v>2.03213743368601</v>
       </c>
       <c r="H233" t="n">
-        <v>0.231858188062383</v>
+        <v>0.231710019946086</v>
       </c>
       <c r="I233" t="n">
         <v>0</v>
       </c>
       <c r="J233" t="n">
-        <v>0.0740049044391601</v>
+        <v>0.0739575986504049</v>
       </c>
       <c r="K233" t="n">
-        <v>-6.69864932905008</v>
+        <v>-6.68097652559757</v>
       </c>
       <c r="L233" t="n">
-        <v>-0.716284523806407</v>
+        <v>-0.715826019352711</v>
       </c>
       <c r="M233" t="n">
         <v>0</v>
@@ -23245,31 +23245,31 @@
         <v>0</v>
       </c>
       <c r="P233" t="n">
-        <v>-0.0683649374505635</v>
+        <v>-0.0683212258677145</v>
       </c>
       <c r="Q233" t="n">
-        <v>-0.0480629733680494</v>
+        <v>-0.0482322018492991</v>
       </c>
       <c r="R233" t="n">
-        <v>0.00020307512422245</v>
+        <v>0.000202945296596091</v>
       </c>
       <c r="S233" t="n">
-        <v>-0.00101704678480214</v>
+        <v>-0.00101639657675773</v>
       </c>
       <c r="T233" t="n">
-        <v>-0.000246262931694933</v>
+        <v>-0.000246105493538782</v>
       </c>
       <c r="U233" t="n">
-        <v>-0.00173873340704849</v>
+        <v>-0.00173762181611431</v>
       </c>
       <c r="V233" t="n">
-        <v>-0.000240713587954182</v>
+        <v>-0.000240559697536508</v>
       </c>
       <c r="W233" t="n">
-        <v>-5.85610569442293</v>
+        <v>-5.91436861463351</v>
       </c>
       <c r="X233" t="n">
-        <v>-0.971363260940978</v>
+        <v>-0.997986039803619</v>
       </c>
       <c r="Y233" t="e">
         <v>#NUM!</v>
@@ -23278,19 +23278,19 @@
         <v>#NUM!</v>
       </c>
       <c r="AA233" t="n">
-        <v>5.83837236134983</v>
+        <v>5.82151809025094</v>
       </c>
       <c r="AB233" t="n">
-        <v>-15.0254389336204</v>
+        <v>-15.1001656021526</v>
       </c>
       <c r="AC233" t="n">
-        <v>-8.26462586715547</v>
+        <v>-8.35404029139007</v>
       </c>
       <c r="AD233" t="n">
         <v>0</v>
       </c>
       <c r="AE233" t="n">
-        <v>-5.3983459691189</v>
+        <v>-5.42295707256856</v>
       </c>
     </row>
     <row r="234">
@@ -23310,19 +23310,19 @@
         <v>#NUM!</v>
       </c>
       <c r="F234" t="n">
-        <v>3.61883779505171</v>
+        <v>3.6008832698024</v>
       </c>
       <c r="G234" t="n">
-        <v>2.01253197286209</v>
+        <v>2.01324124556049</v>
       </c>
       <c r="H234" t="n">
-        <v>0.234557978962108</v>
+        <v>0.234408086220064</v>
       </c>
       <c r="I234" t="n">
         <v>0</v>
       </c>
       <c r="J234" t="n">
-        <v>0.0728476492349111</v>
+        <v>0.0728010830921995</v>
       </c>
       <c r="K234" t="n">
         <v>0</v>
@@ -23340,25 +23340,25 @@
         <v>0</v>
       </c>
       <c r="P234" t="n">
-        <v>-0.0406778993403949</v>
+        <v>-0.0406518917355554</v>
       </c>
       <c r="Q234" t="n">
-        <v>-0.0420127997662854</v>
+        <v>-0.0421545338553969</v>
       </c>
       <c r="R234" t="n">
-        <v>0.00019938519262096</v>
+        <v>0.000199257723950149</v>
       </c>
       <c r="S234" t="n">
-        <v>-0.00102183495765849</v>
+        <v>-0.00102118168850391</v>
       </c>
       <c r="T234" t="n">
         <v>0</v>
       </c>
       <c r="U234" t="n">
-        <v>-0.00170685993997872</v>
+        <v>-0.00170576872623044</v>
       </c>
       <c r="V234" t="n">
-        <v>-0.0000808993597260053</v>
+        <v>-0.0000808476400810527</v>
       </c>
       <c r="W234" t="n">
         <v>0</v>
@@ -23373,13 +23373,13 @@
         <v>#NUM!</v>
       </c>
       <c r="AA234" t="n">
-        <v>5.84186840142057</v>
+        <v>5.82481725337155</v>
       </c>
       <c r="AB234" t="n">
-        <v>-0.0853214219395807</v>
+        <v>-0.0854355399239037</v>
       </c>
       <c r="AC234" t="n">
-        <v>5.76191206134956</v>
+        <v>5.74474043125708</v>
       </c>
       <c r="AD234" t="n">
         <v>0</v>
@@ -23405,19 +23405,19 @@
         <v>#NUM!</v>
       </c>
       <c r="F235" t="n">
-        <v>3.57190915749324</v>
+        <v>3.55419131342856</v>
       </c>
       <c r="G235" t="n">
-        <v>1.99148494947807</v>
+        <v>1.99218795199887</v>
       </c>
       <c r="H235" t="n">
-        <v>0.237042748862387</v>
+        <v>0.236891268974758</v>
       </c>
       <c r="I235" t="n">
         <v>0</v>
       </c>
       <c r="J235" t="n">
-        <v>0.0714050408210611</v>
+        <v>0.0713593967211659</v>
       </c>
       <c r="K235" t="n">
         <v>0</v>
@@ -23435,25 +23435,25 @@
         <v>0</v>
       </c>
       <c r="P235" t="n">
-        <v>-0.0224270681918266</v>
+        <v>-0.0224127298025257</v>
       </c>
       <c r="Q235" t="n">
-        <v>-0.0391679966473345</v>
+        <v>-0.0393082942887716</v>
       </c>
       <c r="R235" t="n">
-        <v>0.000195472164597558</v>
+        <v>0.000195347197630985</v>
       </c>
       <c r="S235" t="n">
-        <v>-0.000602817314630225</v>
+        <v>-0.00060243192778068</v>
       </c>
       <c r="T235" t="n">
         <v>0</v>
       </c>
       <c r="U235" t="n">
-        <v>-0.00134103295066386</v>
+        <v>-0.00134017561449183</v>
       </c>
       <c r="V235" t="n">
-        <v>-0.000079303089971064</v>
+        <v>-0.0000792523907588815</v>
       </c>
       <c r="W235" t="n">
         <v>0</v>
@@ -23468,13 +23468,13 @@
         <v>#NUM!</v>
       </c>
       <c r="AA235" t="n">
-        <v>5.77683544730007</v>
+        <v>5.76000594526847</v>
       </c>
       <c r="AB235" t="n">
-        <v>-0.0634333166754442</v>
+        <v>-0.0635581412121001</v>
       </c>
       <c r="AC235" t="n">
-        <v>5.71735009124706</v>
+        <v>5.70039358694634</v>
       </c>
       <c r="AD235" t="n">
         <v>0</v>
@@ -23500,19 +23500,19 @@
         <v>#NUM!</v>
       </c>
       <c r="F236" t="n">
-        <v>3.53283769353085</v>
+        <v>3.51531773280946</v>
       </c>
       <c r="G236" t="n">
-        <v>1.97295169427431</v>
+        <v>1.97365007397347</v>
       </c>
       <c r="H236" t="n">
-        <v>0.240084864985276</v>
+        <v>0.239931441795108</v>
       </c>
       <c r="I236" t="n">
         <v>0</v>
       </c>
       <c r="J236" t="n">
-        <v>0.0702056512828767</v>
+        <v>0.0701607737628257</v>
       </c>
       <c r="K236" t="n">
         <v>0</v>
@@ -23530,16 +23530,16 @@
         <v>0</v>
       </c>
       <c r="P236" t="n">
-        <v>-0.0220272179875595</v>
+        <v>-0.0220131352469431</v>
       </c>
       <c r="Q236" t="n">
-        <v>-0.0383046594556231</v>
+        <v>-0.0384426166632188</v>
       </c>
       <c r="R236" t="n">
-        <v>0.00019200497056138</v>
+        <v>0.000191882220196571</v>
       </c>
       <c r="S236" t="n">
-        <v>-0.000601315167640283</v>
+        <v>-0.000600930741209028</v>
       </c>
       <c r="T236" t="n">
         <v>0</v>
@@ -23548,7 +23548,7 @@
         <v>0</v>
       </c>
       <c r="V236" t="n">
-        <v>-0.0000778902840891251</v>
+        <v>-0.000077840488093452</v>
       </c>
       <c r="W236" t="n">
         <v>0</v>
@@ -23563,13 +23563,13 @@
         <v>#NUM!</v>
       </c>
       <c r="AA236" t="n">
-        <v>5.7228426053631</v>
+        <v>5.70619759532021</v>
       </c>
       <c r="AB236" t="n">
-        <v>-0.0608283714847691</v>
+        <v>-0.0609519654886842</v>
       </c>
       <c r="AC236" t="n">
-        <v>5.66575878201711</v>
+        <v>5.64898837085382</v>
       </c>
       <c r="AD236" t="n">
         <v>0</v>
@@ -23595,19 +23595,19 @@
         <v>#NUM!</v>
       </c>
       <c r="F237" t="n">
-        <v>3.49051621077527</v>
+        <v>3.47321054898445</v>
       </c>
       <c r="G237" t="n">
-        <v>1.95373257578532</v>
+        <v>1.95442521053282</v>
       </c>
       <c r="H237" t="n">
-        <v>0.234199985229249</v>
+        <v>0.234050321110559</v>
       </c>
       <c r="I237" t="n">
         <v>0</v>
       </c>
       <c r="J237" t="n">
-        <v>0.0688559445108052</v>
+        <v>0.0688119296558737</v>
       </c>
       <c r="K237" t="n">
         <v>0</v>
@@ -23625,16 +23625,16 @@
         <v>0</v>
       </c>
       <c r="P237" t="n">
-        <v>-0.0173222943965292</v>
+        <v>-0.0173112197637809</v>
       </c>
       <c r="Q237" t="n">
-        <v>-0.038621710072626</v>
+        <v>-0.0388104514204572</v>
       </c>
       <c r="R237" t="n">
-        <v>0.000443326345424968</v>
+        <v>0.000443042923254768</v>
       </c>
       <c r="S237" t="n">
-        <v>-0.000601522800031365</v>
+        <v>-0.000601138240837524</v>
       </c>
       <c r="T237" t="n">
         <v>0</v>
@@ -23643,7 +23643,7 @@
         <v>0</v>
       </c>
       <c r="V237" t="n">
-        <v>-0.0000764148755326047</v>
+        <v>-0.0000763660228065846</v>
       </c>
       <c r="W237" t="n">
         <v>0</v>
@@ -23658,13 +23658,13 @@
         <v>#NUM!</v>
       </c>
       <c r="AA237" t="n">
-        <v>5.65636057969709</v>
+        <v>5.6399194780742</v>
       </c>
       <c r="AB237" t="n">
-        <v>-0.0561858713814589</v>
+        <v>-0.056363421790418</v>
       </c>
       <c r="AC237" t="n">
-        <v>5.60359143289177</v>
+        <v>5.58697498436932</v>
       </c>
       <c r="AD237" t="n">
         <v>0</v>
@@ -23696,13 +23696,13 @@
         <v>0</v>
       </c>
       <c r="H238" t="n">
-        <v>0.228596003723281</v>
+        <v>0.228449919265009</v>
       </c>
       <c r="I238" t="n">
         <v>0</v>
       </c>
       <c r="J238" t="n">
-        <v>0.0676872253848881</v>
+        <v>0.0676439575150105</v>
       </c>
       <c r="K238" t="n">
         <v>0</v>
@@ -23723,13 +23723,13 @@
         <v>0</v>
       </c>
       <c r="Q238" t="n">
-        <v>-0.0304767008433723</v>
+        <v>-0.0306265926763216</v>
       </c>
       <c r="R238" t="n">
         <v>0</v>
       </c>
       <c r="S238" t="n">
-        <v>-0.00050252608529723</v>
+        <v>-0.000502204815656503</v>
       </c>
       <c r="T238" t="n">
         <v>0</v>
@@ -23753,13 +23753,13 @@
         <v>#NUM!</v>
       </c>
       <c r="AA238" t="n">
-        <v>0.296118713669662</v>
+        <v>0.295929501370882</v>
       </c>
       <c r="AB238" t="n">
-        <v>-0.0309793896730409</v>
+        <v>-0.0311289610020127</v>
       </c>
       <c r="AC238" t="n">
-        <v>0.265236855801254</v>
+        <v>0.264898522262119</v>
       </c>
       <c r="AD238" t="n">
         <v>0</v>
@@ -23791,13 +23791,13 @@
         <v>0</v>
       </c>
       <c r="H239" t="n">
-        <v>0.222967253161161</v>
+        <v>0.222824764294032</v>
       </c>
       <c r="I239" t="n">
         <v>0</v>
       </c>
       <c r="J239" t="n">
-        <v>0.0665448370139842</v>
+        <v>0.0665022993056748</v>
       </c>
       <c r="K239" t="n">
         <v>0</v>
@@ -23818,13 +23818,13 @@
         <v>0</v>
       </c>
       <c r="Q239" t="n">
-        <v>-0.0290543150850642</v>
+        <v>-0.0292019463996334</v>
       </c>
       <c r="R239" t="n">
         <v>0</v>
       </c>
       <c r="S239" t="n">
-        <v>-0.00039689958062066</v>
+        <v>-0.000396645839132258</v>
       </c>
       <c r="T239" t="n">
         <v>0</v>
@@ -23848,13 +23848,13 @@
         <v>#NUM!</v>
       </c>
       <c r="AA239" t="n">
-        <v>0.289354471356583</v>
+        <v>0.28916957894134</v>
       </c>
       <c r="AB239" t="n">
-        <v>-0.0294513370987211</v>
+        <v>-0.0295987152676964</v>
       </c>
       <c r="AC239" t="n">
-        <v>0.259993658575408</v>
+        <v>0.259661821673705</v>
       </c>
       <c r="AD239" t="n">
         <v>0</v>
@@ -23886,13 +23886,13 @@
         <v>0</v>
       </c>
       <c r="H240" t="n">
-        <v>0.217222991828037</v>
+        <v>0.217084172487286</v>
       </c>
       <c r="I240" t="n">
         <v>0</v>
       </c>
       <c r="J240" t="n">
-        <v>0.0651602323155318</v>
+        <v>0.0651185795937728</v>
       </c>
       <c r="K240" t="n">
         <v>0</v>
@@ -23913,13 +23913,13 @@
         <v>0</v>
       </c>
       <c r="Q240" t="n">
-        <v>-0.028478455978438</v>
+        <v>-0.0286231606348469</v>
       </c>
       <c r="R240" t="n">
         <v>0</v>
       </c>
       <c r="S240" t="n">
-        <v>-0.000293806788589155</v>
+        <v>-0.000293618955169596</v>
       </c>
       <c r="T240" t="n">
         <v>0</v>
@@ -23943,13 +23943,13 @@
         <v>#NUM!</v>
       </c>
       <c r="AA240" t="n">
-        <v>0.282232800105162</v>
+        <v>0.282052456079552</v>
       </c>
       <c r="AB240" t="n">
-        <v>-0.0287723516395919</v>
+        <v>-0.0289168688952376</v>
       </c>
       <c r="AC240" t="n">
-        <v>0.253546744255501</v>
+        <v>0.253222298008468</v>
       </c>
       <c r="AD240" t="n">
         <v>0</v>
@@ -23981,13 +23981,13 @@
         <v>0</v>
       </c>
       <c r="H241" t="n">
-        <v>0.21178474837133</v>
+        <v>0.211649403096106</v>
       </c>
       <c r="I241" t="n">
         <v>0</v>
       </c>
       <c r="J241" t="n">
-        <v>0.0639949553369039</v>
+        <v>0.0639540474155803</v>
       </c>
       <c r="K241" t="n">
         <v>0</v>
@@ -24008,13 +24008,13 @@
         <v>0</v>
       </c>
       <c r="Q241" t="n">
-        <v>-0.0283890131432666</v>
+        <v>-0.0285306772592885</v>
       </c>
       <c r="R241" t="n">
         <v>0</v>
       </c>
       <c r="S241" t="n">
-        <v>-0.000193882328858648</v>
+        <v>-0.000193758378148312</v>
       </c>
       <c r="T241" t="n">
         <v>0</v>
@@ -24038,13 +24038,13 @@
         <v>#NUM!</v>
       </c>
       <c r="AA241" t="n">
-        <v>0.275635721590795</v>
+        <v>0.27545959094879</v>
       </c>
       <c r="AB241" t="n">
-        <v>-0.0285829539138032</v>
+        <v>-0.0287244943582483</v>
       </c>
       <c r="AC241" t="n">
-        <v>0.247136460618288</v>
+        <v>0.246819186118347</v>
       </c>
       <c r="AD241" t="n">
         <v>0</v>
@@ -24103,13 +24103,13 @@
         <v>0</v>
       </c>
       <c r="Q242" t="n">
-        <v>-0.00945491171455536</v>
+        <v>-0.00950251500132452</v>
       </c>
       <c r="R242" t="n">
         <v>0</v>
       </c>
       <c r="S242" t="n">
-        <v>-0.0000968169368454454</v>
+        <v>-0.0000967550409194685</v>
       </c>
       <c r="T242" t="n">
         <v>0</v>
@@ -24136,10 +24136,10 @@
         <v>0</v>
       </c>
       <c r="AB242" t="n">
-        <v>-0.00955173835804979</v>
+        <v>-0.00959927979563127</v>
       </c>
       <c r="AC242" t="n">
-        <v>-0.00955173835804979</v>
+        <v>-0.00959927979563127</v>
       </c>
       <c r="AD242" t="n">
         <v>0</v>
@@ -24198,7 +24198,7 @@
         <v>0</v>
       </c>
       <c r="Q243" t="n">
-        <v>-0.00928811981361368</v>
+        <v>-0.00933488329082626</v>
       </c>
       <c r="R243" t="n">
         <v>0</v>
@@ -24231,10 +24231,10 @@
         <v>0</v>
       </c>
       <c r="AB243" t="n">
-        <v>-0.00928811981361368</v>
+        <v>-0.00933488329082626</v>
       </c>
       <c r="AC243" t="n">
-        <v>-0.00928811981361368</v>
+        <v>-0.00933488329082626</v>
       </c>
       <c r="AD243" t="n">
         <v>0</v>
@@ -24293,7 +24293,7 @@
         <v>0</v>
       </c>
       <c r="Q244" t="n">
-        <v>-0.00910520943664025</v>
+        <v>-0.00915105195514218</v>
       </c>
       <c r="R244" t="n">
         <v>0</v>
@@ -24326,10 +24326,10 @@
         <v>0</v>
       </c>
       <c r="AB244" t="n">
-        <v>-0.00910520943664025</v>
+        <v>-0.00915105195514218</v>
       </c>
       <c r="AC244" t="n">
-        <v>-0.00910520943664025</v>
+        <v>-0.00915105195514218</v>
       </c>
       <c r="AD244" t="n">
         <v>0</v>
@@ -24388,7 +24388,7 @@
         <v>0</v>
       </c>
       <c r="Q245" t="n">
-        <v>-0.00893867002384327</v>
+        <v>-0.00898367400999615</v>
       </c>
       <c r="R245" t="n">
         <v>0</v>
@@ -24421,10 +24421,10 @@
         <v>0</v>
       </c>
       <c r="AB245" t="n">
-        <v>-0.00893867002384327</v>
+        <v>-0.00898367400999615</v>
       </c>
       <c r="AC245" t="n">
-        <v>-0.00893867002384327</v>
+        <v>-0.00898367400999615</v>
       </c>
       <c r="AD245" t="n">
         <v>0</v>

</xml_diff>